<commit_message>
Complete modelling evaluation, Streamlit MVP and report draft
</commit_message>
<xml_diff>
--- a/docs/datasets/data_inventory_catalog.xlsx
+++ b/docs/datasets/data_inventory_catalog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Otros ordenadores\Mi MacBook Pro\HSLU-CAS_ML-CAS Project\swiss-data-intelligence\docs\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4433B21A-1ACF-4D60-8ABE-D9F4B0677CBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD168807-DCA1-42BB-A6F1-8FA0B1807F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-30" windowWidth="38640" windowHeight="21120" xr2:uid="{5C47462E-D134-4FE4-861E-AA4D8B7637EC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{5C47462E-D134-4FE4-861E-AA4D8B7637EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="249">
   <si>
     <t>Dataset ID</t>
   </si>
@@ -439,9 +439,6 @@
     <t>Not directly user-facing; used to translate geographic codes into canton names</t>
   </si>
   <si>
-    <t>Required lookup table for interpreting BFS GEO codes in housing and demographic datasets.</t>
-  </si>
-  <si>
     <t>Original Dataset Name</t>
   </si>
   <si>
@@ -460,9 +457,6 @@
     <t>OCCUPIED_DWELLINGS_BY_OCCUPANCY_STATUS_AND_CANTON</t>
   </si>
   <si>
-    <t>Value</t>
-  </si>
-  <si>
     <t>Occupied Dwellings by Occupancy Status and Canton</t>
   </si>
   <si>
@@ -559,9 +553,6 @@
     <t>DEMOGRAPHIC_BALANCE_BY_CANTON</t>
   </si>
   <si>
-    <t>Provisional demographic balance of the permanent resident population by year, canton, citizenship (category), sex, age and demographic component</t>
-  </si>
-  <si>
     <t>Demographic Balance by Canton</t>
   </si>
   <si>
@@ -574,12 +565,6 @@
     <t>STAT-TAB (BFS PX-Web)</t>
   </si>
   <si>
-    <t>(STAT-TAB URL)</t>
-  </si>
-  <si>
-    <t>(API URL o export URL)</t>
-  </si>
-  <si>
     <t>XLSX (export), JSON (API)</t>
   </si>
   <si>
@@ -589,22 +574,6 @@
     <t>English</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">2025 </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(or selected years via API)</t>
-    </r>
-  </si>
-  <si>
     <t>Canton × Year × Citizenship × Sex × Age × Demographic Component</t>
   </si>
   <si>
@@ -626,65 +595,6 @@
     <t>Year; Canton</t>
   </si>
   <si>
-    <r>
-      <t>RESIDENT_POPULATION_BY_CANTON</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">; </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>HOME_OWNERSHIP_RATE_BY_CANTON</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">; </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>OCCUPIED_DWELLINGS_BY_OCCUPANCY_STATUS_AND_CANTON</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">; </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>CANTON_LOOKUP</t>
-    </r>
-  </si>
-  <si>
     <t>Provides the demographic dynamics of each canton, including births, deaths, immigration, emigration and population changes. Supports population growth analysis and regional comparisons.</t>
   </si>
   <si>
@@ -851,6 +761,20 @@
   </si>
   <si>
     <t xml:space="preserve"> PRIVATE_HOUSEHOLDS_BY_HOUSEHOLD_SIZE </t>
+  </si>
+  <si>
+    <t>Selected</t>
+  </si>
+  <si>
+    <t>Good candidate for MVP.
+Selected as target variable for the MVP analytical dataset.</t>
+  </si>
+  <si>
+    <t>Required lookup table for interpreting BFS GEO codes in housing and demographic datasets.
+Selected as reference data for geographic code and canton-name harmonisation.</t>
+  </si>
+  <si>
+    <t>Evaluated but not selected dataset</t>
   </si>
 </sst>
 </file>
@@ -1370,46 +1294,46 @@
   <cols>
     <col min="1" max="1" width="2.85546875" customWidth="1"/>
     <col min="2" max="2" width="63.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="83.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="74.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="34.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="46.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="57.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="50.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="97.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="45.85546875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="20" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="44.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="26" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="53.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="47.5703125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="27.28515625" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="37.28515625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="24" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="61.85546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="127" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="19" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="38.140625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="61.140625" customWidth="1"/>
+    <col min="40" max="40" width="62.85546875" customWidth="1"/>
     <col min="41" max="41" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="9" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="59.85546875" bestFit="1" customWidth="1"/>
     <col min="44" max="45" width="11.42578125" customWidth="1"/>
     <col min="46" max="16384" width="11.42578125" hidden="1"/>
   </cols>
@@ -1419,7 +1343,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>1</v>
@@ -1542,12 +1466,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="2:43">
+    <row r="3" spans="2:43" ht="25.5">
       <c r="B3" s="14" t="s">
         <v>36</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>16</v>
@@ -1654,28 +1578,28 @@
       <c r="AL3" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="AM3" s="14" t="s">
+      <c r="AM3" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="AN3" s="14" t="s">
+      <c r="AN3" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="AO3" s="14" t="s">
+      <c r="AO3" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="AP3" s="14" t="s">
-        <v>34</v>
+      <c r="AP3" s="16" t="s">
+        <v>245</v>
       </c>
       <c r="AQ3" s="16" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="4" spans="2:43" ht="63.75">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="4" spans="2:43" ht="51">
       <c r="B4" s="14" t="s">
         <v>125</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>126</v>
@@ -1746,22 +1670,24 @@
       <c r="AJ4" s="14"/>
       <c r="AK4" s="14"/>
       <c r="AL4" s="14"/>
-      <c r="AM4" s="14"/>
-      <c r="AN4" s="14" t="s">
+      <c r="AM4" s="16"/>
+      <c r="AN4" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="AO4" s="14"/>
-      <c r="AP4" s="14"/>
+      <c r="AO4" s="16"/>
+      <c r="AP4" s="16" t="s">
+        <v>245</v>
+      </c>
       <c r="AQ4" s="16" t="s">
-        <v>137</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" spans="2:43">
       <c r="B5" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
@@ -1779,7 +1705,7 @@
       </c>
       <c r="L5" s="14"/>
       <c r="M5" s="14" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="N5" s="14"/>
       <c r="O5" s="14"/>
@@ -1806,27 +1732,27 @@
       <c r="AJ5" s="14"/>
       <c r="AK5" s="14"/>
       <c r="AL5" s="14"/>
-      <c r="AM5" s="14"/>
-      <c r="AN5" s="14"/>
-      <c r="AO5" s="14"/>
-      <c r="AP5" s="14"/>
+      <c r="AM5" s="16"/>
+      <c r="AN5" s="16"/>
+      <c r="AO5" s="16"/>
+      <c r="AP5" s="16"/>
       <c r="AQ5" s="16"/>
     </row>
-    <row r="6" spans="2:43" ht="153">
+    <row r="6" spans="2:43" ht="51">
       <c r="B6" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="D6" s="14" t="s">
         <v>143</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>145</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>17</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G6" s="14" t="s">
         <v>23</v>
@@ -1835,22 +1761,22 @@
         <v>20</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="J6" s="14" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="K6" s="14" t="s">
         <v>50</v>
       </c>
       <c r="L6" s="14" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="M6" s="14" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="N6" s="14" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="O6" s="14" t="s">
         <v>19</v>
@@ -1859,7 +1785,7 @@
         <v>30</v>
       </c>
       <c r="Q6" s="14" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="R6" s="14" t="s">
         <v>62</v>
@@ -1874,10 +1800,10 @@
         <v>122</v>
       </c>
       <c r="V6" s="14" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="W6" s="14" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="X6" s="14" t="s">
         <v>77</v>
@@ -1895,66 +1821,66 @@
         <v>6</v>
       </c>
       <c r="AC6" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="AD6" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="AE6" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="AD6" s="14" t="s">
+      <c r="AF6" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="AE6" s="14" t="s">
+      <c r="AG6" s="14" t="s">
         <v>155</v>
-      </c>
-      <c r="AF6" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="AG6" s="14" t="s">
-        <v>157</v>
       </c>
       <c r="AH6" s="14" t="s">
         <v>20</v>
       </c>
       <c r="AI6" s="14" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="AJ6" s="14" t="s">
         <v>20</v>
       </c>
       <c r="AK6" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="AL6" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="AM6" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="AL6" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="AM6" s="14" t="s">
+      <c r="AN6" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="AO6" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="AP6" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="AQ6" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="AN6" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="AO6" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="AP6" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="AQ6" s="16" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="7" spans="2:43" ht="229.5">
+    </row>
+    <row r="7" spans="2:43" ht="76.5">
       <c r="B7" s="14" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>17</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G7" s="14" t="s">
         <v>23</v>
@@ -1963,22 +1889,22 @@
         <v>20</v>
       </c>
       <c r="I7" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="J7" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="M7" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="N7" s="14" t="s">
         <v>167</v>
-      </c>
-      <c r="J7" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="K7" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="L7" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="M7" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="N7" s="14" t="s">
-        <v>169</v>
       </c>
       <c r="O7" s="14" t="s">
         <v>19</v>
@@ -1987,7 +1913,7 @@
         <v>30</v>
       </c>
       <c r="Q7" s="14" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="R7" s="14" t="s">
         <v>62</v>
@@ -2002,10 +1928,10 @@
         <v>122</v>
       </c>
       <c r="V7" s="14" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="W7" s="14" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="X7" s="14" t="s">
         <v>77</v>
@@ -2023,66 +1949,66 @@
         <v>6</v>
       </c>
       <c r="AC7" s="14" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="AD7" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="AE7" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="AF7" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="AE7" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="AF7" s="14" t="s">
-        <v>156</v>
-      </c>
       <c r="AG7" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="AH7" s="14" t="s">
         <v>20</v>
       </c>
       <c r="AI7" s="14" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="AJ7" s="14" t="s">
         <v>20</v>
       </c>
       <c r="AK7" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="AL7" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="AM7" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="AM7" s="16" t="s">
+        <v>170</v>
+      </c>
+      <c r="AN7" s="16" t="s">
+        <v>171</v>
+      </c>
+      <c r="AO7" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="AP7" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="AQ7" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="AN7" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="AO7" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="AP7" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="AQ7" s="16" t="s">
+    </row>
+    <row r="8" spans="2:43" ht="63.75">
+      <c r="B8" s="14" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="8" spans="2:43" ht="204">
-      <c r="B8" s="14" t="s">
+      <c r="C8" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="E8" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="C8" s="14" t="s">
-        <v>202</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>179</v>
-      </c>
       <c r="F8" s="14" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G8" s="14" t="s">
         <v>23</v>
@@ -2091,31 +2017,31 @@
         <v>20</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="K8" s="14" t="s">
         <v>50</v>
       </c>
       <c r="L8" s="14" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="M8" s="14" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="N8" s="14" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="O8" s="14" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="P8" s="14" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="Q8" s="14" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="R8" s="14" t="s">
         <v>62</v>
@@ -2127,150 +2053,150 @@
         <v>68</v>
       </c>
       <c r="U8" s="14" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="V8" s="14" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="W8" s="14" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="X8" s="14" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="Y8" s="14" t="s">
         <v>77</v>
       </c>
       <c r="Z8" s="14" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="AA8" s="14" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="AB8" s="14" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="AC8" s="14" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="AD8" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="AE8" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="AF8" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="AE8" s="14" t="s">
-        <v>194</v>
-      </c>
-      <c r="AF8" s="14" t="s">
-        <v>200</v>
-      </c>
       <c r="AG8" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="AH8" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="AI8" s="14" t="s">
         <v>20</v>
       </c>
       <c r="AJ8" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="AK8" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="AL8" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="AM8" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="AM8" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="AN8" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="AO8" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="AP8" s="16" t="s">
+        <v>248</v>
+      </c>
+      <c r="AQ8" s="16" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="9" spans="2:43" ht="38.25">
+      <c r="B9" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="AN8" s="14" t="s">
+      <c r="C9" s="14" t="s">
+        <v>206</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>207</v>
+      </c>
+      <c r="E9" s="14" t="s">
         <v>197</v>
       </c>
-      <c r="AO8" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="AP8" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="AQ8" s="16" t="s">
+      <c r="F9" s="14" t="s">
+        <v>208</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="H9" s="14" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="9" spans="2:43" ht="140.25">
-      <c r="B9" s="14" t="s">
+      <c r="I9" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="J9" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="K9" s="14" t="s">
+        <v>211</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>200</v>
+      </c>
+      <c r="M9" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="N9" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="O9" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="P9" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q9" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="R9" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="S9" s="14" t="s">
+        <v>202</v>
+      </c>
+      <c r="T9" s="14" t="s">
         <v>203</v>
       </c>
-      <c r="C9" s="14" t="s">
-        <v>213</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>214</v>
-      </c>
-      <c r="E9" s="14" t="s">
+      <c r="U9" s="14" t="s">
+        <v>217</v>
+      </c>
+      <c r="V9" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="W9" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="X9" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="F9" s="14" t="s">
-        <v>215</v>
-      </c>
-      <c r="G9" s="14" t="s">
-        <v>216</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="I9" s="14" t="s">
-        <v>217</v>
-      </c>
-      <c r="J9" s="14" t="s">
-        <v>206</v>
-      </c>
-      <c r="K9" s="14" t="s">
-        <v>218</v>
-      </c>
-      <c r="L9" s="14" t="s">
-        <v>207</v>
-      </c>
-      <c r="M9" s="14" t="s">
-        <v>219</v>
-      </c>
-      <c r="N9" s="14" t="s">
+      <c r="Y9" s="14" t="s">
+        <v>204</v>
+      </c>
+      <c r="Z9" s="14" t="s">
         <v>220</v>
-      </c>
-      <c r="O9" s="14" t="s">
-        <v>221</v>
-      </c>
-      <c r="P9" s="14" t="s">
-        <v>222</v>
-      </c>
-      <c r="Q9" s="14" t="s">
-        <v>223</v>
-      </c>
-      <c r="R9" s="14" t="s">
-        <v>208</v>
-      </c>
-      <c r="S9" s="14" t="s">
-        <v>209</v>
-      </c>
-      <c r="T9" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="U9" s="14" t="s">
-        <v>224</v>
-      </c>
-      <c r="V9" s="14" t="s">
-        <v>225</v>
-      </c>
-      <c r="W9" s="14" t="s">
-        <v>226</v>
-      </c>
-      <c r="X9" s="14" t="s">
-        <v>211</v>
-      </c>
-      <c r="Y9" s="14" t="s">
-        <v>211</v>
-      </c>
-      <c r="Z9" s="14" t="s">
-        <v>227</v>
       </c>
       <c r="AA9" s="14">
         <v>3.024</v>
@@ -2279,126 +2205,126 @@
         <v>107</v>
       </c>
       <c r="AC9" s="14" t="s">
+        <v>221</v>
+      </c>
+      <c r="AD9" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="AE9" s="14" t="s">
+        <v>223</v>
+      </c>
+      <c r="AF9" s="14" t="s">
+        <v>224</v>
+      </c>
+      <c r="AG9" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="AH9" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="AI9" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="AJ9" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="AK9" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="AL9" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="AM9" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="AN9" s="16" t="s">
+        <v>227</v>
+      </c>
+      <c r="AO9" s="16" t="s">
         <v>228</v>
       </c>
-      <c r="AD9" s="14" t="s">
+      <c r="AP9" s="16" t="s">
+        <v>205</v>
+      </c>
+      <c r="AQ9" s="16" t="s">
         <v>229</v>
       </c>
-      <c r="AE9" s="14" t="s">
+    </row>
+    <row r="10" spans="2:43" ht="38.25">
+      <c r="B10" s="14" t="s">
+        <v>244</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>230</v>
       </c>
-      <c r="AF9" s="14" t="s">
+      <c r="D10" s="14" t="s">
         <v>231</v>
       </c>
-      <c r="AG9" s="14" t="s">
+      <c r="E10" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="F10" s="14" t="s">
         <v>232</v>
       </c>
-      <c r="AH9" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AI9" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AJ9" s="14" t="s">
-        <v>232</v>
-      </c>
-      <c r="AK9" s="14" t="s">
-        <v>232</v>
-      </c>
-      <c r="AL9" s="14" t="s">
-        <v>232</v>
-      </c>
-      <c r="AM9" s="14" t="s">
+      <c r="G10" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="J10" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="K10" s="14" t="s">
+        <v>211</v>
+      </c>
+      <c r="L10" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="AN9" s="14" t="s">
+      <c r="M10" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="AO9" s="14" t="s">
+      <c r="N10" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="O10" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="P10" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q10" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="R10" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="S10" s="14" t="s">
+        <v>202</v>
+      </c>
+      <c r="T10" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="U10" s="14" t="s">
+        <v>217</v>
+      </c>
+      <c r="V10" s="14" t="s">
         <v>235</v>
       </c>
-      <c r="AP9" s="14" t="s">
-        <v>212</v>
-      </c>
-      <c r="AQ9" s="16" t="s">
+      <c r="W10" s="14" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="10" spans="2:43" ht="127.5">
-      <c r="B10" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="C10" s="14" t="s">
+      <c r="X10" s="14" t="s">
+        <v>204</v>
+      </c>
+      <c r="Y10" s="14" t="s">
+        <v>204</v>
+      </c>
+      <c r="Z10" s="14" t="s">
         <v>237</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>238</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>204</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>239</v>
-      </c>
-      <c r="G10" s="14" t="s">
-        <v>216</v>
-      </c>
-      <c r="H10" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="I10" s="14" t="s">
-        <v>217</v>
-      </c>
-      <c r="J10" s="14" t="s">
-        <v>206</v>
-      </c>
-      <c r="K10" s="14" t="s">
-        <v>218</v>
-      </c>
-      <c r="L10" s="14" t="s">
-        <v>240</v>
-      </c>
-      <c r="M10" s="14" t="s">
-        <v>241</v>
-      </c>
-      <c r="N10" s="14" t="s">
-        <v>220</v>
-      </c>
-      <c r="O10" s="14" t="s">
-        <v>221</v>
-      </c>
-      <c r="P10" s="14" t="s">
-        <v>222</v>
-      </c>
-      <c r="Q10" s="14" t="s">
-        <v>223</v>
-      </c>
-      <c r="R10" s="14" t="s">
-        <v>208</v>
-      </c>
-      <c r="S10" s="14" t="s">
-        <v>209</v>
-      </c>
-      <c r="T10" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="U10" s="14" t="s">
-        <v>224</v>
-      </c>
-      <c r="V10" s="14" t="s">
-        <v>242</v>
-      </c>
-      <c r="W10" s="14" t="s">
-        <v>243</v>
-      </c>
-      <c r="X10" s="14" t="s">
-        <v>211</v>
-      </c>
-      <c r="Y10" s="14" t="s">
-        <v>211</v>
-      </c>
-      <c r="Z10" s="14" t="s">
-        <v>244</v>
       </c>
       <c r="AA10" s="14">
         <v>1.1339999999999999</v>
@@ -2407,52 +2333,52 @@
         <v>26</v>
       </c>
       <c r="AC10" s="14" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="AD10" s="14" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="AE10" s="14" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="AF10" s="14" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="AG10" s="14" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="AH10" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="AI10" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="AJ10" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="AK10" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="AL10" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="AM10" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="AN10" s="16" t="s">
+        <v>242</v>
+      </c>
+      <c r="AO10" s="16" t="s">
+        <v>228</v>
+      </c>
+      <c r="AP10" s="16" t="s">
         <v>205</v>
       </c>
-      <c r="AI10" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AJ10" s="14" t="s">
-        <v>232</v>
-      </c>
-      <c r="AK10" s="14" t="s">
-        <v>232</v>
-      </c>
-      <c r="AL10" s="14" t="s">
-        <v>232</v>
-      </c>
-      <c r="AM10" s="14" t="s">
-        <v>248</v>
-      </c>
-      <c r="AN10" s="14" t="s">
-        <v>249</v>
-      </c>
-      <c r="AO10" s="14" t="s">
-        <v>235</v>
-      </c>
-      <c r="AP10" s="14" t="s">
-        <v>212</v>
-      </c>
       <c r="AQ10" s="16" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="11" spans="2:43" ht="204">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="11" spans="2:43">
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
@@ -2496,7 +2422,7 @@
       <c r="AP11" s="14"/>
       <c r="AQ11" s="16"/>
     </row>
-    <row r="12" spans="2:43" ht="204">
+    <row r="12" spans="2:43">
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
@@ -2540,7 +2466,7 @@
       <c r="AP12" s="14"/>
       <c r="AQ12" s="16"/>
     </row>
-    <row r="13" spans="2:43" ht="204">
+    <row r="13" spans="2:43">
       <c r="B13" s="14"/>
       <c r="C13" s="14"/>
       <c r="D13" s="14"/>
@@ -2584,7 +2510,7 @@
       <c r="AP13" s="14"/>
       <c r="AQ13" s="16"/>
     </row>
-    <row r="14" spans="2:43" ht="204">
+    <row r="14" spans="2:43">
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
       <c r="D14" s="14"/>
@@ -2628,7 +2554,7 @@
       <c r="AP14" s="14"/>
       <c r="AQ14" s="16"/>
     </row>
-    <row r="15" spans="2:43" ht="204">
+    <row r="15" spans="2:43">
       <c r="B15" s="14"/>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
@@ -2672,7 +2598,7 @@
       <c r="AP15" s="14"/>
       <c r="AQ15" s="16"/>
     </row>
-    <row r="16" spans="2:43" ht="204">
+    <row r="16" spans="2:43">
       <c r="B16" s="14"/>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
@@ -2716,7 +2642,7 @@
       <c r="AP16" s="14"/>
       <c r="AQ16" s="16"/>
     </row>
-    <row r="17" spans="2:43" ht="204">
+    <row r="17" spans="2:43">
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
       <c r="D17" s="14"/>
@@ -2760,7 +2686,7 @@
       <c r="AP17" s="14"/>
       <c r="AQ17" s="16"/>
     </row>
-    <row r="18" spans="2:43" ht="204">
+    <row r="18" spans="2:43">
       <c r="B18" s="14"/>
       <c r="C18" s="14"/>
       <c r="D18" s="14"/>
@@ -2804,7 +2730,7 @@
       <c r="AP18" s="14"/>
       <c r="AQ18" s="16"/>
     </row>
-    <row r="19" spans="2:43" ht="204">
+    <row r="19" spans="2:43">
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
       <c r="D19" s="14"/>
@@ -3377,604 +3303,264 @@
       <c r="AQ31" s="11"/>
     </row>
     <row r="32" spans="2:43">
-      <c r="B32" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="C32" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="D32" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="F32" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="G32" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="H32" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I32" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="J32" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="K32" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="L32" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M32" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="N32" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="O32" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="P32" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q32" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="R32" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="S32" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="T32" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="U32" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="V32" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="W32" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="X32" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="Y32" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="Z32" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="AA32" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="AB32" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AC32" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="AD32" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="AE32" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="AF32" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="AG32" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="AH32" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="AI32" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="AJ32" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="AK32" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="AL32" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="AM32" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="AN32" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="AO32" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="AP32" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="AQ32" s="11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="33" spans="2:43" ht="255">
-      <c r="B33" s="12" t="s">
-        <v>176</v>
-      </c>
-      <c r="C33" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="D33" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="E33" s="10" t="s">
-        <v>179</v>
-      </c>
-      <c r="F33" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="G33" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="H33" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="I33" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="J33" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="K33" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="L33" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="M33" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="N33" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="O33" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="P33" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="Q33" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="R33" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="S33" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="T33" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="U33" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="V33" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="W33" s="10" t="s">
-        <v>189</v>
-      </c>
-      <c r="X33" s="10" t="s">
-        <v>190</v>
-      </c>
-      <c r="Y33" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="Z33" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="AA33" s="10" t="s">
-        <v>191</v>
-      </c>
-      <c r="AB33" s="10" t="s">
-        <v>192</v>
-      </c>
-      <c r="AC33" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="AD33" s="12" t="s">
-        <v>193</v>
-      </c>
-      <c r="AE33" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="AF33" s="12" t="s">
-        <v>195</v>
-      </c>
-      <c r="AG33" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="AH33" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="AI33" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="AJ33" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="AK33" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="AL33" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="AM33" s="10" t="s">
-        <v>196</v>
-      </c>
-      <c r="AN33" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="AO33" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="AP33" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="AQ33" s="10" t="s">
-        <v>198</v>
-      </c>
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="11"/>
+      <c r="I32" s="11"/>
+      <c r="J32" s="11"/>
+      <c r="K32" s="11"/>
+      <c r="L32" s="11"/>
+      <c r="M32" s="11"/>
+      <c r="N32" s="11"/>
+      <c r="O32" s="11"/>
+      <c r="P32" s="11"/>
+      <c r="Q32" s="11"/>
+      <c r="R32" s="11"/>
+      <c r="S32" s="11"/>
+      <c r="T32" s="11"/>
+      <c r="U32" s="11"/>
+      <c r="V32" s="11"/>
+      <c r="W32" s="11"/>
+      <c r="X32" s="11"/>
+      <c r="Y32" s="11"/>
+      <c r="Z32" s="11"/>
+      <c r="AA32" s="11"/>
+      <c r="AB32" s="11"/>
+      <c r="AC32" s="11"/>
+      <c r="AD32" s="11"/>
+      <c r="AE32" s="11"/>
+      <c r="AF32" s="11"/>
+      <c r="AG32" s="11"/>
+      <c r="AH32" s="11"/>
+      <c r="AI32" s="11"/>
+      <c r="AJ32" s="11"/>
+      <c r="AK32" s="11"/>
+      <c r="AL32" s="11"/>
+      <c r="AM32" s="11"/>
+      <c r="AN32" s="11"/>
+      <c r="AO32" s="11"/>
+      <c r="AP32" s="11"/>
+      <c r="AQ32" s="11"/>
+    </row>
+    <row r="33" spans="2:43">
+      <c r="B33" s="12"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10"/>
+      <c r="K33" s="10"/>
+      <c r="L33" s="13"/>
+      <c r="M33" s="13"/>
+      <c r="N33" s="10"/>
+      <c r="O33" s="10"/>
+      <c r="P33" s="10"/>
+      <c r="Q33" s="10"/>
+      <c r="R33" s="10"/>
+      <c r="S33" s="10"/>
+      <c r="T33" s="10"/>
+      <c r="U33" s="10"/>
+      <c r="V33" s="10"/>
+      <c r="W33" s="10"/>
+      <c r="X33" s="10"/>
+      <c r="Y33" s="10"/>
+      <c r="Z33" s="10"/>
+      <c r="AA33" s="10"/>
+      <c r="AB33" s="10"/>
+      <c r="AC33" s="10"/>
+      <c r="AD33" s="12"/>
+      <c r="AE33" s="12"/>
+      <c r="AF33" s="12"/>
+      <c r="AG33" s="10"/>
+      <c r="AH33" s="10"/>
+      <c r="AI33" s="10"/>
+      <c r="AJ33" s="10"/>
+      <c r="AK33" s="10"/>
+      <c r="AL33" s="10"/>
+      <c r="AM33" s="10"/>
+      <c r="AN33" s="10"/>
+      <c r="AO33" s="10"/>
+      <c r="AP33" s="10"/>
+      <c r="AQ33" s="10"/>
     </row>
     <row r="36" spans="2:43">
-      <c r="B36" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>144</v>
-      </c>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
     </row>
     <row r="37" spans="2:43">
-      <c r="B37" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="C37" s="12" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="38" spans="2:43" ht="60">
-      <c r="B38" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="C38" s="10" t="s">
-        <v>177</v>
-      </c>
+      <c r="B37" s="11"/>
+      <c r="C37" s="12"/>
+    </row>
+    <row r="38" spans="2:43">
+      <c r="B38" s="11"/>
+      <c r="C38" s="10"/>
     </row>
     <row r="39" spans="2:43">
-      <c r="B39" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="C39" s="10" t="s">
-        <v>178</v>
-      </c>
+      <c r="B39" s="11"/>
+      <c r="C39" s="10"/>
     </row>
     <row r="40" spans="2:43">
-      <c r="B40" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="C40" s="10" t="s">
-        <v>179</v>
-      </c>
+      <c r="B40" s="11"/>
+      <c r="C40" s="10"/>
     </row>
     <row r="41" spans="2:43">
-      <c r="B41" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C41" s="10" t="s">
-        <v>180</v>
-      </c>
+      <c r="B41" s="11"/>
+      <c r="C41" s="10"/>
     </row>
     <row r="42" spans="2:43">
-      <c r="B42" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C42" s="10" t="s">
-        <v>23</v>
-      </c>
+      <c r="B42" s="11"/>
+      <c r="C42" s="10"/>
     </row>
     <row r="43" spans="2:43">
-      <c r="B43" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C43" s="10" t="s">
-        <v>20</v>
-      </c>
+      <c r="B43" s="11"/>
+      <c r="C43" s="10"/>
     </row>
     <row r="44" spans="2:43">
-      <c r="B44" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="C44" s="10" t="s">
-        <v>167</v>
-      </c>
+      <c r="B44" s="11"/>
+      <c r="C44" s="10"/>
     </row>
     <row r="45" spans="2:43">
-      <c r="B45" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C45" s="10" t="s">
-        <v>181</v>
-      </c>
+      <c r="B45" s="11"/>
+      <c r="C45" s="10"/>
     </row>
     <row r="46" spans="2:43">
-      <c r="B46" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C46" s="10" t="s">
-        <v>50</v>
-      </c>
+      <c r="B46" s="11"/>
+      <c r="C46" s="10"/>
     </row>
     <row r="47" spans="2:43">
-      <c r="B47" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C47" s="13" t="s">
-        <v>182</v>
-      </c>
+      <c r="B47" s="11"/>
+      <c r="C47" s="13"/>
     </row>
     <row r="48" spans="2:43">
-      <c r="B48" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C48" s="13" t="s">
-        <v>183</v>
-      </c>
+      <c r="B48" s="11"/>
+      <c r="C48" s="13"/>
     </row>
     <row r="49" spans="2:3">
-      <c r="B49" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C49" s="10" t="s">
-        <v>149</v>
-      </c>
+      <c r="B49" s="11"/>
+      <c r="C49" s="10"/>
     </row>
     <row r="50" spans="2:3">
-      <c r="B50" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C50" s="10" t="s">
-        <v>184</v>
-      </c>
+      <c r="B50" s="11"/>
+      <c r="C50" s="10"/>
     </row>
     <row r="51" spans="2:3">
-      <c r="B51" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C51" s="10" t="s">
-        <v>185</v>
-      </c>
+      <c r="B51" s="11"/>
+      <c r="C51" s="10"/>
     </row>
     <row r="52" spans="2:3">
-      <c r="B52" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C52" s="10" t="s">
-        <v>186</v>
-      </c>
+      <c r="B52" s="11"/>
+      <c r="C52" s="10"/>
     </row>
     <row r="53" spans="2:3">
-      <c r="B53" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C53" s="10" t="s">
-        <v>62</v>
-      </c>
+      <c r="B53" s="11"/>
+      <c r="C53" s="10"/>
     </row>
     <row r="54" spans="2:3">
-      <c r="B54" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="C54" s="10" t="s">
-        <v>65</v>
-      </c>
+      <c r="B54" s="11"/>
+      <c r="C54" s="10"/>
     </row>
     <row r="55" spans="2:3">
-      <c r="B55" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C55" s="10" t="s">
-        <v>68</v>
-      </c>
+      <c r="B55" s="11"/>
+      <c r="C55" s="10"/>
     </row>
     <row r="56" spans="2:3">
-      <c r="B56" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C56" s="10" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="57" spans="2:3" ht="30">
-      <c r="B57" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C57" s="10" t="s">
-        <v>188</v>
-      </c>
+      <c r="B56" s="11"/>
+      <c r="C56" s="10"/>
+    </row>
+    <row r="57" spans="2:3">
+      <c r="B57" s="11"/>
+      <c r="C57" s="10"/>
     </row>
     <row r="58" spans="2:3">
-      <c r="B58" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="C58" s="10" t="s">
-        <v>189</v>
-      </c>
+      <c r="B58" s="11"/>
+      <c r="C58" s="10"/>
     </row>
     <row r="59" spans="2:3">
-      <c r="B59" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="C59" s="10" t="s">
-        <v>190</v>
-      </c>
+      <c r="B59" s="11"/>
+      <c r="C59" s="10"/>
     </row>
     <row r="60" spans="2:3">
-      <c r="B60" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="C60" s="10" t="s">
-        <v>77</v>
-      </c>
+      <c r="B60" s="11"/>
+      <c r="C60" s="10"/>
     </row>
     <row r="61" spans="2:3">
-      <c r="B61" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="C61" s="10" t="s">
-        <v>158</v>
-      </c>
+      <c r="B61" s="11"/>
+      <c r="C61" s="10"/>
     </row>
     <row r="62" spans="2:3">
-      <c r="B62" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="C62" s="10" t="s">
-        <v>191</v>
-      </c>
+      <c r="B62" s="11"/>
+      <c r="C62" s="10"/>
     </row>
     <row r="63" spans="2:3">
-      <c r="B63" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="C63" s="10" t="s">
-        <v>192</v>
-      </c>
+      <c r="B63" s="11"/>
+      <c r="C63" s="10"/>
     </row>
     <row r="64" spans="2:3">
-      <c r="B64" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="C64" s="10" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="65" spans="2:3" ht="25.5">
-      <c r="B65" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C65" s="12" t="s">
-        <v>193</v>
-      </c>
+      <c r="B64" s="11"/>
+      <c r="C64" s="10"/>
+    </row>
+    <row r="65" spans="2:3">
+      <c r="B65" s="11"/>
+      <c r="C65" s="12"/>
     </row>
     <row r="66" spans="2:3">
-      <c r="B66" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="C66" s="12" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="67" spans="2:3" ht="57.75">
-      <c r="B67" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="C67" s="12" t="s">
-        <v>195</v>
-      </c>
+      <c r="B66" s="11"/>
+      <c r="C66" s="12"/>
+    </row>
+    <row r="67" spans="2:3">
+      <c r="B67" s="11"/>
+      <c r="C67" s="12"/>
     </row>
     <row r="68" spans="2:3">
-      <c r="B68" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="C68" s="10" t="s">
-        <v>157</v>
-      </c>
+      <c r="B68" s="11"/>
+      <c r="C68" s="10"/>
     </row>
     <row r="69" spans="2:3">
-      <c r="B69" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="C69" s="10" t="s">
-        <v>157</v>
-      </c>
+      <c r="B69" s="11"/>
+      <c r="C69" s="10"/>
     </row>
     <row r="70" spans="2:3">
-      <c r="B70" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="C70" s="10" t="s">
-        <v>20</v>
-      </c>
+      <c r="B70" s="11"/>
+      <c r="C70" s="10"/>
     </row>
     <row r="71" spans="2:3">
-      <c r="B71" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="C71" s="10" t="s">
-        <v>157</v>
-      </c>
+      <c r="B71" s="11"/>
+      <c r="C71" s="10"/>
     </row>
     <row r="72" spans="2:3">
-      <c r="B72" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="C72" s="10" t="s">
-        <v>157</v>
-      </c>
+      <c r="B72" s="11"/>
+      <c r="C72" s="10"/>
     </row>
     <row r="73" spans="2:3">
-      <c r="B73" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C73" s="10" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="74" spans="2:3" ht="75">
-      <c r="B74" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C74" s="10" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="75" spans="2:3" ht="90">
-      <c r="B75" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C75" s="10" t="s">
-        <v>197</v>
-      </c>
+      <c r="B73" s="11"/>
+      <c r="C73" s="10"/>
+    </row>
+    <row r="74" spans="2:3">
+      <c r="B74" s="11"/>
+      <c r="C74" s="10"/>
+    </row>
+    <row r="75" spans="2:3">
+      <c r="B75" s="11"/>
+      <c r="C75" s="10"/>
     </row>
     <row r="76" spans="2:3">
-      <c r="B76" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="C76" s="10" t="s">
-        <v>118</v>
-      </c>
+      <c r="B76" s="11"/>
+      <c r="C76" s="10"/>
     </row>
     <row r="77" spans="2:3">
-      <c r="B77" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C77" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="78" spans="2:3" ht="105">
-      <c r="B78" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C78" s="10" t="s">
-        <v>198</v>
-      </c>
+      <c r="B77" s="11"/>
+      <c r="C77" s="10"/>
+    </row>
+    <row r="78" spans="2:3">
+      <c r="B78" s="11"/>
+      <c r="C78" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>